<commit_message>
chore(ag): filter sheet in statistics, improve templates
</commit_message>
<xml_diff>
--- a/django/camac/statistics/config/kt_ag/dossiers_municipality.xlsx
+++ b/django/camac/statistics/config/kt_ag/dossiers_municipality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5D048F-4086-4349-B39F-4BA2046CA4EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5295B004-DFD0-4BB6-8F16-B3D18A017CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="31755" windowHeight="16770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13245" yWindow="2400" windowWidth="23415" windowHeight="12705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="13" r:id="rId4"/>
+    <pivotCache cacheId="48" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>Dossier-Nr.</t>
   </si>
@@ -67,9 +67,6 @@
     <t>Dauer</t>
   </si>
   <si>
-    <t>Anzahl</t>
-  </si>
-  <si>
     <t>&lt;= 70 Tage</t>
   </si>
   <si>
@@ -88,9 +85,6 @@
     <t>Zeilenbeschriftungen</t>
   </si>
   <si>
-    <t>Anzahl von Dossier-Nr.</t>
-  </si>
-  <si>
     <t>(Leer)</t>
   </si>
   <si>
@@ -98,6 +92,12 @@
   </si>
   <si>
     <t>Anteil</t>
+  </si>
+  <si>
+    <t>Anzahl Dossiers</t>
+  </si>
+  <si>
+    <t>Anzahl Gesuche nach Gesuchstyp</t>
   </si>
 </sst>
 </file>
@@ -107,7 +107,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +145,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -219,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -236,10 +243,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -258,7 +266,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46111.659267476854" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="8" xr:uid="{7F2E8BCB-6429-4F29-B162-7F5B0E97F404}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46121.734951041668" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="16" xr:uid="{7F2E8BCB-6429-4F29-B162-7F5B0E97F404}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G1048576" sheet="Data"/>
   </cacheSource>
@@ -297,7 +305,79 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="8">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="16">
+  <r>
+    <m/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
   <r>
     <m/>
     <x v="0"/>
@@ -374,7 +454,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EDA4FBB-689F-4687-8A8A-191B1E09B9C1}" name="PivotTable1" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EDA4FBB-689F-4687-8A8A-191B1E09B9C1}" name="PivotTable1" cacheId="48" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField dataField="1" showAll="0"/>
@@ -406,7 +486,7 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Anzahl von Dossier-Nr." fld="0" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Anzahl Dossiers" fld="0" subtotal="count" baseField="1" baseItem="1"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -829,6 +909,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -841,54 +923,54 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="5">
         <f>COUNTIF(Data!G:G,"&lt;=70")</f>
         <v>0</v>
       </c>
-      <c r="C4" s="15" t="e">
+      <c r="C4" s="14" t="e">
         <f>COUNTIF(Data!G:G,"&lt;=70") / $B$7</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTIFS(Data!G:G,"&gt;70",Data!G:G,"&lt;=100")</f>
         <v>0</v>
       </c>
-      <c r="C5" s="16" t="e">
+      <c r="C5" s="15" t="e">
         <f>COUNTIFS(Data!G:G,"&gt;70",Data!G:G,"&lt;=100") / $B$7</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="8">
         <f>COUNTIF(Data!G:G,"&gt;100")</f>
         <v>0</v>
       </c>
-      <c r="C6" s="17" t="e">
+      <c r="C6" s="16" t="e">
         <f>COUNTIF(Data!G:G,"&gt;100") / $B$7</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="3">
         <f>SUM(B4:B6)</f>
@@ -903,37 +985,40 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1309E224-DB63-4B75-BDE8-A0B093978349}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" s="18"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="14"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="14"/>
+      <c r="B5" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -941,17 +1026,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5e238f3b-cf1c-4dc8-b1c3-14677632393c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="fb274a4b-4ecf-4ae2-a446-66548455045d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -960,7 +1034,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D7FFFCF5F95BC94D9B7DF34B9D0CF76C" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="a8184ac6384f947bbc55bc4d9e1749d1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5e238f3b-cf1c-4dc8-b1c3-14677632393c" xmlns:ns3="a7360a35-2516-4210-888a-7cc8dd0a384d" xmlns:ns4="fb274a4b-4ecf-4ae2-a446-66548455045d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6dc33f40212c2dffa236803017f7661f" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="5e238f3b-cf1c-4dc8-b1c3-14677632393c"/>
@@ -1200,18 +1274,18 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5e238f3b-cf1c-4dc8-b1c3-14677632393c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="fb274a4b-4ecf-4ae2-a446-66548455045d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1358810-D270-4430-A211-3ABFE193427A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5e238f3b-cf1c-4dc8-b1c3-14677632393c"/>
-    <ds:schemaRef ds:uri="fb274a4b-4ecf-4ae2-a446-66548455045d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16F88CF8-4776-46E4-AB0C-41B3C8FC9322}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1219,7 +1293,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{898C8B08-FCC0-41BA-BCBB-BC205106FBDF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1237,4 +1311,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1358810-D270-4430-A211-3ABFE193427A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5e238f3b-cf1c-4dc8-b1c3-14677632393c"/>
+    <ds:schemaRef ds:uri="fb274a4b-4ecf-4ae2-a446-66548455045d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(ag): add export-date to all sheet, updated templates and labels
</commit_message>
<xml_diff>
--- a/django/camac/statistics/config/kt_ag/dossiers_municipality.xlsx
+++ b/django/camac/statistics/config/kt_ag/dossiers_municipality.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5295B004-DFD0-4BB6-8F16-B3D18A017CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A094193E-0C3F-44D5-B6AD-5E447638B6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13245" yWindow="2400" windowWidth="23415" windowHeight="12705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7275" yWindow="3480" windowWidth="28800" windowHeight="14925" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="48" r:id="rId4"/>
+    <pivotCache cacheId="77" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -142,6 +142,7 @@
       <b/>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -150,8 +151,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
+      <sz val="14"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -246,8 +246,8 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -266,7 +266,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46121.734951041668" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="16" xr:uid="{7F2E8BCB-6429-4F29-B162-7F5B0E97F404}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46136.444819791664" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="16" xr:uid="{7F2E8BCB-6429-4F29-B162-7F5B0E97F404}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G1048576" sheet="Data"/>
   </cacheSource>
@@ -454,8 +454,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EDA4FBB-689F-4687-8A8A-191B1E09B9C1}" name="PivotTable1" cacheId="48" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EDA4FBB-689F-4687-8A8A-191B1E09B9C1}" name="PivotTable1" cacheId="77" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A5:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField dataField="1" showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
@@ -905,7 +905,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -918,65 +918,65 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B6" s="5">
         <f>COUNTIF(Data!G:G,"&lt;=70")</f>
         <v>0</v>
       </c>
-      <c r="C4" s="14" t="e">
-        <f>COUNTIF(Data!G:G,"&lt;=70") / $B$7</f>
+      <c r="C6" s="14" t="e">
+        <f>COUNTIF(Data!G:G,"&lt;=70") / $B$9</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B7" s="6">
         <f>COUNTIFS(Data!G:G,"&gt;70",Data!G:G,"&lt;=100")</f>
         <v>0</v>
       </c>
-      <c r="C5" s="15" t="e">
-        <f>COUNTIFS(Data!G:G,"&gt;70",Data!G:G,"&lt;=100") / $B$7</f>
+      <c r="C7" s="15" t="e">
+        <f>COUNTIFS(Data!G:G,"&gt;70",Data!G:G,"&lt;=100") / $B$9</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B8" s="8">
         <f>COUNTIF(Data!G:G,"&gt;100")</f>
         <v>0</v>
       </c>
-      <c r="C6" s="16" t="e">
-        <f>COUNTIF(Data!G:G,"&gt;100") / $B$7</f>
+      <c r="C8" s="16" t="e">
+        <f>COUNTIF(Data!G:G,"&gt;100") / $B$9</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3">
-        <f>SUM(B4:B6)</f>
+      <c r="B9" s="3">
+        <f>SUM(B6:B8)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -985,40 +985,40 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1309E224-DB63-4B75-BDE8-A0B093978349}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
         <v>19</v>
       </c>
       <c r="F1" s="11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="18"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="B6" s="17"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="18"/>
+      <c r="B7" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1026,15 +1026,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D7FFFCF5F95BC94D9B7DF34B9D0CF76C" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="a8184ac6384f947bbc55bc4d9e1749d1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5e238f3b-cf1c-4dc8-b1c3-14677632393c" xmlns:ns3="a7360a35-2516-4210-888a-7cc8dd0a384d" xmlns:ns4="fb274a4b-4ecf-4ae2-a446-66548455045d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6dc33f40212c2dffa236803017f7661f" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="5e238f3b-cf1c-4dc8-b1c3-14677632393c"/>
@@ -1274,6 +1265,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1286,14 +1286,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16F88CF8-4776-46E4-AB0C-41B3C8FC9322}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{898C8B08-FCC0-41BA-BCBB-BC205106FBDF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1313,6 +1305,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16F88CF8-4776-46E4-AB0C-41B3C8FC9322}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1358810-D270-4430-A211-3ABFE193427A}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
chore(ag): update statistics template - deadline value
</commit_message>
<xml_diff>
--- a/django/camac/statistics/config/kt_ag/dossiers_municipality.xlsx
+++ b/django/camac/statistics/config/kt_ag/dossiers_municipality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A094193E-0C3F-44D5-B6AD-5E447638B6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC06583-3683-486F-A4EC-65EB5C9AF033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7275" yWindow="3480" windowWidth="28800" windowHeight="14925" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="33105" windowHeight="17610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="77" r:id="rId4"/>
+    <pivotCache cacheId="4" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -70,9 +70,6 @@
     <t>&lt;= 70 Tage</t>
   </si>
   <si>
-    <t>71 - 100 Tage</t>
-  </si>
-  <si>
     <t>&gt; 100 Tage</t>
   </si>
   <si>
@@ -98,6 +95,9 @@
   </si>
   <si>
     <t>Anzahl Gesuche nach Gesuchstyp</t>
+  </si>
+  <si>
+    <t>&lt;= 100 Tage</t>
   </si>
 </sst>
 </file>
@@ -246,8 +246,8 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -266,7 +266,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46136.444819791664" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="16" xr:uid="{7F2E8BCB-6429-4F29-B162-7F5B0E97F404}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46146.649407986108" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="16" xr:uid="{7F2E8BCB-6429-4F29-B162-7F5B0E97F404}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:G1048576" sheet="Data"/>
   </cacheSource>
@@ -454,7 +454,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EDA4FBB-689F-4687-8A8A-191B1E09B9C1}" name="PivotTable1" cacheId="77" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EDA4FBB-689F-4687-8A8A-191B1E09B9C1}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField dataField="1" showAll="0"/>
@@ -923,10 +923,10 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -944,20 +944,20 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIFS(Data!G:G,"&gt;70",Data!G:G,"&lt;=100")</f>
+        <f>COUNTIF(Data!G:G,"&lt;=100")</f>
         <v>0</v>
       </c>
       <c r="C7" s="15" t="e">
-        <f>COUNTIFS(Data!G:G,"&gt;70",Data!G:G,"&lt;=100") / $B$9</f>
+        <f>COUNTIF(Data!G:G,"&lt;=100") / $B$9</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="8">
         <f>COUNTIF(Data!G:G,"&gt;100")</f>
@@ -970,10 +970,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="3">
-        <f>SUM(B6:B8)</f>
+        <f>SUM(B7:B8)</f>
         <v>0</v>
       </c>
       <c r="C9" s="3"/>
@@ -993,32 +993,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
-        <v>19</v>
+      <c r="A1" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="17"/>
+        <v>14</v>
+      </c>
+      <c r="B6" s="18"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="17"/>
+        <v>15</v>
+      </c>
+      <c r="B7" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>